<commit_message>
Auto backup 2026-06-30 09:05:01
</commit_message>
<xml_diff>
--- a/SwissTechShehzad/27-06-2026/27-06-2026.xlsx
+++ b/SwissTechShehzad/27-06-2026/27-06-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\27-06-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23DD1CA-24F1-463F-98B5-437DD68CE68C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C59B44-301E-4E4B-B156-3F1CB27C77E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1905" windowWidth="29040" windowHeight="17520" xr2:uid="{8BCFAE85-CB20-435D-AEB6-6494F3D318DE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="210">
   <si>
     <t>Sr No</t>
   </si>
@@ -634,6 +634,39 @@
   </si>
   <si>
     <t>mightyape.co.nz</t>
+  </si>
+  <si>
+    <t>noelleeming.co.nz</t>
+  </si>
+  <si>
+    <t>rubbermonkey.co.nz</t>
+  </si>
+  <si>
+    <t>elive.co.nz</t>
+  </si>
+  <si>
+    <t>photogear.co.nz</t>
+  </si>
+  <si>
+    <t>priceme.co.nz</t>
+  </si>
+  <si>
+    <t>einfo.co.nz</t>
+  </si>
+  <si>
+    <t>heathcotes.co.nz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website </t>
+  </si>
+  <si>
+    <t>bestbuy.com</t>
+  </si>
+  <si>
+    <t>walmart.com</t>
+  </si>
+  <si>
+    <t>newegg.com</t>
   </si>
 </sst>
 </file>
@@ -737,13 +770,217 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="67">
+  <dxfs count="87">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1744,17 +1981,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55654141-CD25-4A03-806C-27730D60093D}">
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:H167"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="5.8984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="94" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.59765625" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="6.8984375" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="11.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1773,8 +2012,14 @@
       <c r="F1" s="1" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1787,14 +2032,20 @@
       <c r="D2" s="4">
         <v>50</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="4">
         <v>59</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2" t="s">
+        <v>207</v>
+      </c>
+      <c r="H2">
+        <v>64.900000000000006</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1807,14 +2058,14 @@
       <c r="D3" s="4">
         <v>2868.7</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="4" t="s">
         <v>171</v>
       </c>
       <c r="F3" s="7">
         <v>2868.7</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:8">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1827,14 +2078,20 @@
       <c r="D4" s="4">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="4">
         <v>34.99</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H4">
+        <v>38.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1847,14 +2104,20 @@
       <c r="D5" s="4">
         <v>678</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="4">
         <v>899</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5" t="s">
+        <v>209</v>
+      </c>
+      <c r="H5">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1867,14 +2130,20 @@
       <c r="D6" s="4">
         <v>38</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="4">
         <v>45.17</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H6">
+        <v>32.49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1887,14 +2156,20 @@
       <c r="D7" s="4">
         <v>297.99</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="4">
         <v>348</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7" t="s">
+        <v>207</v>
+      </c>
+      <c r="H7">
+        <v>191.54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1907,14 +2182,20 @@
       <c r="D8" s="4">
         <v>139.94999999999999</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="4">
         <v>168</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8" t="s">
+        <v>207</v>
+      </c>
+      <c r="H8">
+        <v>109.99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1927,14 +2208,14 @@
       <c r="D9" s="4">
         <v>16999</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="4" t="s">
         <v>171</v>
       </c>
       <c r="F9" s="7">
         <v>15651.3</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:8">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1947,14 +2228,20 @@
       <c r="D10" s="4">
         <v>65</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="4">
         <v>113.85</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10" t="s">
+        <v>209</v>
+      </c>
+      <c r="H10">
+        <v>109.49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1967,14 +2254,20 @@
       <c r="D11" s="4">
         <v>148</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="4">
         <v>168</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="G11" t="s">
+        <v>207</v>
+      </c>
+      <c r="H11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1987,14 +2280,20 @@
       <c r="D12" s="4">
         <v>139.94999999999999</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="4">
         <v>168</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="G12" t="s">
+        <v>207</v>
+      </c>
+      <c r="H12">
+        <v>109.99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -2007,14 +2306,14 @@
       <c r="D13" s="4">
         <v>269</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="4">
         <v>575</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:8">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -2027,14 +2326,20 @@
       <c r="D14" s="4">
         <v>169</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="4">
         <v>179</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
+      <c r="G14" t="s">
+        <v>209</v>
+      </c>
+      <c r="H14">
+        <v>239.95</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -2047,14 +2352,20 @@
       <c r="D15" s="4">
         <v>119</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="4">
         <v>129</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
+      <c r="G15" t="s">
+        <v>208</v>
+      </c>
+      <c r="H15">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -2067,14 +2378,20 @@
       <c r="D16" s="4">
         <v>397</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="4">
         <v>422.36</v>
       </c>
-    </row>
-    <row r="17" spans="1:6">
+      <c r="G16" t="s">
+        <v>207</v>
+      </c>
+      <c r="H16">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -2087,14 +2404,20 @@
       <c r="D17" s="4">
         <v>554</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="4">
         <v>848</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
+      <c r="G17" t="s">
+        <v>207</v>
+      </c>
+      <c r="H17">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -2107,14 +2430,20 @@
       <c r="D18" s="4">
         <v>1299</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="4" t="s">
         <v>191</v>
       </c>
       <c r="F18" s="8">
         <v>1699</v>
       </c>
-    </row>
-    <row r="19" spans="1:6">
+      <c r="G18" t="s">
+        <v>207</v>
+      </c>
+      <c r="H18">
+        <v>1099.99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -2127,14 +2456,20 @@
       <c r="D19" s="4">
         <v>609.4</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="4">
         <v>641.48</v>
       </c>
-    </row>
-    <row r="20" spans="1:6">
+      <c r="G19" t="s">
+        <v>207</v>
+      </c>
+      <c r="H19">
+        <v>399.99</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -2147,14 +2482,20 @@
       <c r="D20" s="4">
         <v>5149</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="4" t="s">
         <v>197</v>
       </c>
       <c r="F20" s="7">
         <v>5658.99</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
+      <c r="G20" t="s">
+        <v>208</v>
+      </c>
+      <c r="H20">
+        <v>3699</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -2167,14 +2508,20 @@
       <c r="D21" s="4">
         <v>249</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="4">
         <v>197.98</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
+      <c r="G21" t="s">
+        <v>208</v>
+      </c>
+      <c r="H21">
+        <v>129.94999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -2187,14 +2534,20 @@
       <c r="D22" s="4">
         <v>249</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="4">
         <v>197.98</v>
       </c>
-    </row>
-    <row r="23" spans="1:6">
+      <c r="G22" t="s">
+        <v>208</v>
+      </c>
+      <c r="H22">
+        <v>129.94999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -2207,14 +2560,14 @@
       <c r="D23" s="4">
         <v>10799</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="4" t="s">
         <v>197</v>
       </c>
       <c r="F23" s="7">
         <v>12668.99</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:8">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -2227,14 +2580,20 @@
       <c r="D24" s="4">
         <v>105</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="4">
         <v>112</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
+      <c r="G24" t="s">
+        <v>208</v>
+      </c>
+      <c r="H24">
+        <v>79.95</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -2247,8 +2606,20 @@
       <c r="D25" s="4">
         <v>119</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
+      <c r="E25" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F25" s="4">
+        <v>141</v>
+      </c>
+      <c r="G25" t="s">
+        <v>207</v>
+      </c>
+      <c r="H25">
+        <v>93.99</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -2261,8 +2632,20 @@
       <c r="D26" s="4">
         <v>119</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
+      <c r="E26" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F26" s="4">
+        <v>141</v>
+      </c>
+      <c r="G26" t="s">
+        <v>207</v>
+      </c>
+      <c r="H26">
+        <v>93.99</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -2275,8 +2658,20 @@
       <c r="D27" s="4">
         <v>119</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
+      <c r="E27" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F27" s="4">
+        <v>141</v>
+      </c>
+      <c r="G27" t="s">
+        <v>207</v>
+      </c>
+      <c r="H27">
+        <v>93.99</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -2289,8 +2684,20 @@
       <c r="D28" s="4">
         <v>119</v>
       </c>
-    </row>
-    <row r="29" spans="1:6">
+      <c r="E28" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F28" s="4">
+        <v>141</v>
+      </c>
+      <c r="G28" t="s">
+        <v>207</v>
+      </c>
+      <c r="H28">
+        <v>93.99</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2303,8 +2710,20 @@
       <c r="D29" s="4">
         <v>187</v>
       </c>
-    </row>
-    <row r="30" spans="1:6">
+      <c r="E29" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F29" s="4">
+        <v>268</v>
+      </c>
+      <c r="G29" t="s">
+        <v>208</v>
+      </c>
+      <c r="H29">
+        <v>158.79</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2317,8 +2736,20 @@
       <c r="D30" s="4">
         <v>195</v>
       </c>
-    </row>
-    <row r="31" spans="1:6">
+      <c r="E30" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F30" s="4">
+        <v>229</v>
+      </c>
+      <c r="G30" t="s">
+        <v>208</v>
+      </c>
+      <c r="H30">
+        <v>175.95</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2331,8 +2762,20 @@
       <c r="D31" s="4">
         <v>229.99</v>
       </c>
-    </row>
-    <row r="32" spans="1:6">
+      <c r="E31" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F31" s="4">
+        <v>339</v>
+      </c>
+      <c r="G31" t="s">
+        <v>207</v>
+      </c>
+      <c r="H31">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2345,8 +2788,20 @@
       <c r="D32" s="4">
         <v>229.99</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="E32" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F32" s="4">
+        <v>339</v>
+      </c>
+      <c r="G32" t="s">
+        <v>207</v>
+      </c>
+      <c r="H32">
+        <v>179.99</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2359,8 +2814,20 @@
       <c r="D33" s="4">
         <v>628</v>
       </c>
-    </row>
-    <row r="34" spans="1:4">
+      <c r="E33" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F33" s="4">
+        <v>657.59</v>
+      </c>
+      <c r="G33" t="s">
+        <v>207</v>
+      </c>
+      <c r="H33">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2373,8 +2840,20 @@
       <c r="D34" s="4">
         <v>688</v>
       </c>
-    </row>
-    <row r="35" spans="1:4">
+      <c r="E34" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F34" s="4">
+        <v>720.32</v>
+      </c>
+      <c r="G34" t="s">
+        <v>208</v>
+      </c>
+      <c r="H34">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2387,8 +2866,20 @@
       <c r="D35" s="4">
         <v>114</v>
       </c>
-    </row>
-    <row r="36" spans="1:4">
+      <c r="E35" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F35" s="4">
+        <v>141</v>
+      </c>
+      <c r="G35" t="s">
+        <v>208</v>
+      </c>
+      <c r="H35">
+        <v>93.95</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2401,8 +2892,20 @@
       <c r="D36" s="4">
         <v>209</v>
       </c>
-    </row>
-    <row r="37" spans="1:4">
+      <c r="E36" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F36" s="4">
+        <v>257.17</v>
+      </c>
+      <c r="G36" t="s">
+        <v>209</v>
+      </c>
+      <c r="H36">
+        <v>149.99</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2415,8 +2918,20 @@
       <c r="D37" s="4">
         <v>187</v>
       </c>
-    </row>
-    <row r="38" spans="1:4">
+      <c r="E37" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F37" s="4">
+        <v>268</v>
+      </c>
+      <c r="G37" t="s">
+        <v>208</v>
+      </c>
+      <c r="H37">
+        <v>158.79</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2429,8 +2944,20 @@
       <c r="D38" s="4">
         <v>629</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
+      <c r="E38" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F38" s="4">
+        <v>730.77</v>
+      </c>
+      <c r="G38" t="s">
+        <v>208</v>
+      </c>
+      <c r="H38">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2443,8 +2970,20 @@
       <c r="D39" s="4">
         <v>485</v>
       </c>
-    </row>
-    <row r="40" spans="1:4">
+      <c r="E39" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F39" s="4">
+        <v>689.99</v>
+      </c>
+      <c r="G39" t="s">
+        <v>208</v>
+      </c>
+      <c r="H39">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2457,8 +2996,20 @@
       <c r="D40" s="4">
         <v>188</v>
       </c>
-    </row>
-    <row r="41" spans="1:4">
+      <c r="E40" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F40" s="4">
+        <v>268</v>
+      </c>
+      <c r="G40" t="s">
+        <v>208</v>
+      </c>
+      <c r="H40">
+        <v>199.95</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -2471,8 +3022,20 @@
       <c r="D41" s="4">
         <v>9299</v>
       </c>
-    </row>
-    <row r="42" spans="1:4">
+      <c r="E41" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F41" s="4">
+        <v>8955.65</v>
+      </c>
+      <c r="G41" t="s">
+        <v>208</v>
+      </c>
+      <c r="H41">
+        <v>6999</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2485,8 +3048,20 @@
       <c r="D42" s="4">
         <v>349.99</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
+      <c r="E42" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F42" s="4">
+        <v>347.1</v>
+      </c>
+      <c r="G42" t="s">
+        <v>208</v>
+      </c>
+      <c r="H42">
+        <v>249.95</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2499,8 +3074,20 @@
       <c r="D43" s="4">
         <v>769</v>
       </c>
-    </row>
-    <row r="44" spans="1:4">
+      <c r="E43" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F43" s="4">
+        <v>1005.94</v>
+      </c>
+      <c r="G43" t="s">
+        <v>208</v>
+      </c>
+      <c r="H43">
+        <v>569.99</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2513,8 +3100,20 @@
       <c r="D44" s="4">
         <v>188</v>
       </c>
-    </row>
-    <row r="45" spans="1:4">
+      <c r="E44" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F44" s="4">
+        <v>268</v>
+      </c>
+      <c r="G44" t="s">
+        <v>208</v>
+      </c>
+      <c r="H44">
+        <v>229.99</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2527,8 +3126,20 @@
       <c r="D45" s="4">
         <v>1349</v>
       </c>
-    </row>
-    <row r="46" spans="1:4">
+      <c r="E45" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F45" s="4">
+        <v>1455.42</v>
+      </c>
+      <c r="G45" t="s">
+        <v>208</v>
+      </c>
+      <c r="H45">
+        <v>1394.29</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2537,8 +3148,20 @@
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
-    </row>
-    <row r="47" spans="1:4">
+      <c r="E46" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F46" s="4">
+        <v>736.47</v>
+      </c>
+      <c r="G46" t="s">
+        <v>208</v>
+      </c>
+      <c r="H46">
+        <v>399.99</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2551,8 +3174,20 @@
       <c r="D47" s="4">
         <v>629</v>
       </c>
-    </row>
-    <row r="48" spans="1:4">
+      <c r="E47" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F47" s="4">
+        <v>730.77</v>
+      </c>
+      <c r="G47" t="s">
+        <v>207</v>
+      </c>
+      <c r="H47">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2565,8 +3200,20 @@
       <c r="D48" s="4">
         <v>2464</v>
       </c>
-    </row>
-    <row r="49" spans="1:4">
+      <c r="E48" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F48" s="4">
+        <v>4255</v>
+      </c>
+      <c r="G48" t="s">
+        <v>208</v>
+      </c>
+      <c r="H48">
+        <v>2799</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2579,8 +3226,20 @@
       <c r="D49" s="4">
         <v>392</v>
       </c>
-    </row>
-    <row r="50" spans="1:4">
+      <c r="E49" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="F49" s="4">
+        <v>689</v>
+      </c>
+      <c r="G49" t="s">
+        <v>208</v>
+      </c>
+      <c r="H49">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2593,8 +3252,20 @@
       <c r="D50" s="4">
         <v>579</v>
       </c>
-    </row>
-    <row r="51" spans="1:4">
+      <c r="E50" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F50" s="4">
+        <v>849</v>
+      </c>
+      <c r="G50" t="s">
+        <v>207</v>
+      </c>
+      <c r="H50">
+        <v>328.99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2607,8 +3278,20 @@
       <c r="D51" s="4">
         <v>88</v>
       </c>
-    </row>
-    <row r="52" spans="1:4">
+      <c r="E51" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F51" s="4">
+        <v>119</v>
+      </c>
+      <c r="G51" t="s">
+        <v>208</v>
+      </c>
+      <c r="H51">
+        <v>89.99</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2621,8 +3304,20 @@
       <c r="D52" s="4">
         <v>409</v>
       </c>
-    </row>
-    <row r="53" spans="1:4">
+      <c r="E52" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F52" s="4">
+        <v>829</v>
+      </c>
+      <c r="G52" t="s">
+        <v>208</v>
+      </c>
+      <c r="H52">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2631,8 +3326,20 @@
       </c>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
-    </row>
-    <row r="54" spans="1:4">
+      <c r="E53" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F53" s="4">
+        <v>688.85</v>
+      </c>
+      <c r="G53" t="s">
+        <v>208</v>
+      </c>
+      <c r="H53">
+        <v>379.99</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -2645,8 +3352,20 @@
       <c r="D54" s="4">
         <v>718</v>
       </c>
-    </row>
-    <row r="55" spans="1:4">
+      <c r="E54" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F54" s="4">
+        <v>730.77</v>
+      </c>
+      <c r="G54" t="s">
+        <v>208</v>
+      </c>
+      <c r="H54">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -2659,8 +3378,14 @@
       <c r="D55" s="4">
         <v>94</v>
       </c>
-    </row>
-    <row r="56" spans="1:4">
+      <c r="E55" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F55" s="4">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -2673,8 +3398,14 @@
       <c r="D56" s="4">
         <v>89.96</v>
       </c>
-    </row>
-    <row r="57" spans="1:4">
+      <c r="E56" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F56" s="4">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -2687,8 +3418,14 @@
       <c r="D57" s="4">
         <v>397</v>
       </c>
-    </row>
-    <row r="58" spans="1:4">
+      <c r="E57" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F57" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -2697,8 +3434,14 @@
       </c>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-    </row>
-    <row r="59" spans="1:4">
+      <c r="E58" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F58" s="4">
+        <v>1164.94</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -2711,8 +3454,14 @@
       <c r="D59" s="4">
         <v>1379</v>
       </c>
-    </row>
-    <row r="60" spans="1:4">
+      <c r="E59" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F59" s="4">
+        <v>2011.35</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -2725,8 +3474,14 @@
       <c r="D60" s="4">
         <v>6399</v>
       </c>
-    </row>
-    <row r="61" spans="1:4">
+      <c r="E60" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F60" s="4">
+        <v>7599</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -2739,8 +3494,14 @@
       <c r="D61" s="4">
         <v>79</v>
       </c>
-    </row>
-    <row r="62" spans="1:4">
+      <c r="E61" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F61" s="4">
+        <v>87.36</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -2753,8 +3514,14 @@
       <c r="D62" s="4">
         <v>79</v>
       </c>
-    </row>
-    <row r="63" spans="1:4">
+      <c r="E62" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F62" s="4">
+        <v>87.36</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -2767,8 +3534,14 @@
       <c r="D63" s="4">
         <v>79</v>
       </c>
-    </row>
-    <row r="64" spans="1:4">
+      <c r="E63" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F63" s="4">
+        <v>87.36</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -2781,8 +3554,14 @@
       <c r="D64" s="4">
         <v>79</v>
       </c>
-    </row>
-    <row r="65" spans="1:4">
+      <c r="E64" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F64" s="4">
+        <v>87.36</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -2795,8 +3574,14 @@
       <c r="D65" s="4">
         <v>79</v>
       </c>
-    </row>
-    <row r="66" spans="1:4">
+      <c r="E65" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F65" s="4">
+        <v>87.36</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -2809,8 +3594,14 @@
       <c r="D66" s="4">
         <v>79</v>
       </c>
-    </row>
-    <row r="67" spans="1:4">
+      <c r="E66" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F66" s="4">
+        <v>87.36</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -2823,8 +3614,14 @@
       <c r="D67" s="4">
         <v>79</v>
       </c>
-    </row>
-    <row r="68" spans="1:4">
+      <c r="E67" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F67" s="4">
+        <v>87.36</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -2837,8 +3634,14 @@
       <c r="D68" s="4">
         <v>79</v>
       </c>
-    </row>
-    <row r="69" spans="1:4">
+      <c r="E68" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F68" s="4">
+        <v>87.36</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -2851,8 +3654,14 @@
       <c r="D69" s="4">
         <v>1859</v>
       </c>
-    </row>
-    <row r="70" spans="1:4">
+      <c r="E69" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="F69" s="4">
+        <v>2638.56</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -2865,8 +3674,14 @@
       <c r="D70" s="4">
         <v>337</v>
       </c>
-    </row>
-    <row r="71" spans="1:4">
+      <c r="E70" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F70" s="4">
+        <v>352.06</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -2879,8 +3694,14 @@
       <c r="D71" s="4">
         <v>879</v>
       </c>
-    </row>
-    <row r="72" spans="1:4">
+      <c r="E71" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F71" s="4">
+        <v>1269</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -2893,8 +3714,14 @@
       <c r="D72" s="4">
         <v>1528</v>
       </c>
-    </row>
-    <row r="73" spans="1:4">
+      <c r="E72" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="F72" s="4">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -2907,8 +3734,14 @@
       <c r="D73" s="4">
         <v>88</v>
       </c>
-    </row>
-    <row r="74" spans="1:4">
+      <c r="E73" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F73" s="4">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -2921,8 +3754,14 @@
       <c r="D74" s="4">
         <v>79</v>
       </c>
-    </row>
-    <row r="75" spans="1:4">
+      <c r="E74" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F74" s="4">
+        <v>87.36</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -2935,8 +3774,14 @@
       <c r="D75" s="4">
         <v>528</v>
       </c>
-    </row>
-    <row r="76" spans="1:4">
+      <c r="E75" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F75" s="4">
+        <v>470.3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -2945,8 +3790,10 @@
       </c>
       <c r="C76" s="4"/>
       <c r="D76" s="4"/>
-    </row>
-    <row r="77" spans="1:4">
+      <c r="E76" s="4"/>
+      <c r="F76" s="4"/>
+    </row>
+    <row r="77" spans="1:6">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -2959,8 +3806,14 @@
       <c r="D77" s="4">
         <v>35</v>
       </c>
-    </row>
-    <row r="78" spans="1:4">
+      <c r="E77" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F77" s="4">
+        <v>40.54</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -2973,8 +3826,14 @@
       <c r="D78" s="4">
         <v>35</v>
       </c>
-    </row>
-    <row r="79" spans="1:4">
+      <c r="E78" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F78" s="4">
+        <v>40.54</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -2987,8 +3846,14 @@
       <c r="D79" s="4">
         <v>35</v>
       </c>
-    </row>
-    <row r="80" spans="1:4">
+      <c r="E79" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F79" s="4">
+        <v>40.54</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -3001,8 +3866,14 @@
       <c r="D80" s="4">
         <v>488</v>
       </c>
-    </row>
-    <row r="81" spans="1:4">
+      <c r="E80" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="F80" s="4">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -3011,8 +3882,10 @@
       </c>
       <c r="C81" s="4"/>
       <c r="D81" s="4"/>
-    </row>
-    <row r="82" spans="1:4">
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+    </row>
+    <row r="82" spans="1:6">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -3025,8 +3898,14 @@
       <c r="D82" s="4">
         <v>1127</v>
       </c>
-    </row>
-    <row r="83" spans="1:4">
+      <c r="E82" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="F82" s="4">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -3039,8 +3918,14 @@
       <c r="D83" s="4">
         <v>698</v>
       </c>
-    </row>
-    <row r="84" spans="1:4">
+      <c r="E83" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F83" s="4">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -3053,8 +3938,14 @@
       <c r="D84" s="4">
         <v>35</v>
       </c>
-    </row>
-    <row r="85" spans="1:4">
+      <c r="E84" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F84" s="4">
+        <v>40.54</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -3067,8 +3958,14 @@
       <c r="D85" s="4">
         <v>35</v>
       </c>
-    </row>
-    <row r="86" spans="1:4">
+      <c r="E85" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F85" s="4">
+        <v>40.54</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -3081,8 +3978,14 @@
       <c r="D86" s="4">
         <v>337</v>
       </c>
-    </row>
-    <row r="87" spans="1:4">
+      <c r="E86" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F86" s="4">
+        <v>383.42</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -3095,8 +3998,14 @@
       <c r="D87" s="4">
         <v>337</v>
       </c>
-    </row>
-    <row r="88" spans="1:4">
+      <c r="E87" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F87" s="4">
+        <v>383.42</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -3109,8 +4018,14 @@
       <c r="D88" s="4">
         <v>404</v>
       </c>
-    </row>
-    <row r="89" spans="1:4">
+      <c r="E88" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F88" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -3123,8 +4038,14 @@
       <c r="D89" s="4">
         <v>349.99</v>
       </c>
-    </row>
-    <row r="90" spans="1:4">
+      <c r="E89" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F89" s="4">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -3137,8 +4058,12 @@
       <c r="D90" s="4">
         <v>337</v>
       </c>
-    </row>
-    <row r="91" spans="1:4">
+      <c r="E90" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F90" s="4"/>
+    </row>
+    <row r="91" spans="1:6">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -3151,8 +4076,14 @@
       <c r="D91" s="4">
         <v>718</v>
       </c>
-    </row>
-    <row r="92" spans="1:4">
+      <c r="E91" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F91" s="4">
+        <v>730.77</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -3161,8 +4092,10 @@
       </c>
       <c r="C92" s="4"/>
       <c r="D92" s="4"/>
-    </row>
-    <row r="93" spans="1:4">
+      <c r="E92" s="4"/>
+      <c r="F92" s="4"/>
+    </row>
+    <row r="93" spans="1:6">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -3175,8 +4108,14 @@
       <c r="D93" s="4">
         <v>527</v>
       </c>
-    </row>
-    <row r="94" spans="1:4">
+      <c r="E93" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F93" s="4">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -3189,8 +4128,14 @@
       <c r="D94" s="4">
         <v>185</v>
       </c>
-    </row>
-    <row r="95" spans="1:4">
+      <c r="E94" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F94" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -3203,8 +4148,14 @@
       <c r="D95" s="4">
         <v>185</v>
       </c>
-    </row>
-    <row r="96" spans="1:4">
+      <c r="E95" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F95" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -3217,8 +4168,14 @@
       <c r="D96" s="4">
         <v>129</v>
       </c>
-    </row>
-    <row r="97" spans="1:4">
+      <c r="E96" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F96" s="4">
+        <v>137.33000000000001</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -3231,8 +4188,14 @@
       <c r="D97" s="4">
         <v>398</v>
       </c>
-    </row>
-    <row r="98" spans="1:4">
+      <c r="E97" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F97" s="4">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -3241,8 +4204,14 @@
       </c>
       <c r="C98" s="4"/>
       <c r="D98" s="4"/>
-    </row>
-    <row r="99" spans="1:4">
+      <c r="E98" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F98" s="4">
+        <v>1289.51</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -3251,8 +4220,10 @@
       </c>
       <c r="C99" s="4"/>
       <c r="D99" s="4"/>
-    </row>
-    <row r="100" spans="1:4">
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+    </row>
+    <row r="100" spans="1:6">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -3265,8 +4236,14 @@
       <c r="D100" s="4">
         <v>239</v>
       </c>
-    </row>
-    <row r="101" spans="1:4">
+      <c r="E100" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F100" s="4">
+        <v>315.23</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -3275,8 +4252,14 @@
       </c>
       <c r="C101" s="4"/>
       <c r="D101" s="4"/>
-    </row>
-    <row r="102" spans="1:4">
+      <c r="E101" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F101" s="4">
+        <v>2914.2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -3285,8 +4268,14 @@
       </c>
       <c r="C102" s="4"/>
       <c r="D102" s="4"/>
-    </row>
-    <row r="103" spans="1:4">
+      <c r="E102" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F102" s="4">
+        <v>1928.14</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -3299,8 +4288,14 @@
       <c r="D103" s="4">
         <v>1195</v>
       </c>
-    </row>
-    <row r="104" spans="1:4">
+      <c r="E103" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F103" s="4">
+        <v>1347.98</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -3309,8 +4304,14 @@
       </c>
       <c r="C104" s="4"/>
       <c r="D104" s="4"/>
-    </row>
-    <row r="105" spans="1:4">
+      <c r="E104" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F104" s="4">
+        <v>1169.69</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -3319,8 +4320,14 @@
       </c>
       <c r="C105" s="4"/>
       <c r="D105" s="4"/>
-    </row>
-    <row r="106" spans="1:4">
+      <c r="E105" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F105" s="4">
+        <v>2748.99</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -3333,8 +4340,14 @@
       <c r="D106" s="4">
         <v>498</v>
       </c>
-    </row>
-    <row r="107" spans="1:4">
+      <c r="E106" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="F106" s="4">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -3347,8 +4360,14 @@
       <c r="D107" s="4">
         <v>598</v>
       </c>
-    </row>
-    <row r="108" spans="1:4">
+      <c r="E107" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F107" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -3361,8 +4380,14 @@
       <c r="D108" s="4">
         <v>598</v>
       </c>
-    </row>
-    <row r="109" spans="1:4">
+      <c r="E108" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F108" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -3371,8 +4396,10 @@
       </c>
       <c r="C109" s="4"/>
       <c r="D109" s="4"/>
-    </row>
-    <row r="110" spans="1:4">
+      <c r="E109" s="4"/>
+      <c r="F109" s="4"/>
+    </row>
+    <row r="110" spans="1:6">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -3381,8 +4408,12 @@
       </c>
       <c r="C110" s="4"/>
       <c r="D110" s="4"/>
-    </row>
-    <row r="111" spans="1:4">
+      <c r="E110" s="4"/>
+      <c r="F110" s="4">
+        <v>1436.35</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -3395,8 +4426,14 @@
       <c r="D111" s="4">
         <v>35</v>
       </c>
-    </row>
-    <row r="112" spans="1:4">
+      <c r="E111" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F111" s="4">
+        <v>40.54</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -3409,8 +4446,14 @@
       <c r="D112" s="4">
         <v>598</v>
       </c>
-    </row>
-    <row r="113" spans="1:4">
+      <c r="E112" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F112" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -3423,8 +4466,14 @@
       <c r="D113" s="4">
         <v>249</v>
       </c>
-    </row>
-    <row r="114" spans="1:4">
+      <c r="E113" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F113" s="4">
+        <v>315.23</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -3433,8 +4482,10 @@
       </c>
       <c r="C114" s="4"/>
       <c r="D114" s="4"/>
-    </row>
-    <row r="115" spans="1:4">
+      <c r="E114" s="4"/>
+      <c r="F114" s="4"/>
+    </row>
+    <row r="115" spans="1:6">
       <c r="A115" s="2">
         <v>114</v>
       </c>
@@ -3447,8 +4498,10 @@
       <c r="D115" s="4">
         <v>1209</v>
       </c>
-    </row>
-    <row r="116" spans="1:4">
+      <c r="E115" s="4"/>
+      <c r="F115" s="4"/>
+    </row>
+    <row r="116" spans="1:6">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -3461,8 +4514,14 @@
       <c r="D116" s="4">
         <v>428</v>
       </c>
-    </row>
-    <row r="117" spans="1:4">
+      <c r="E116" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F116" s="4">
+        <v>616.64</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -3475,8 +4534,14 @@
       <c r="D117" s="4">
         <v>674.79</v>
       </c>
-    </row>
-    <row r="118" spans="1:4">
+      <c r="E117" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F117" s="4">
+        <v>782.56</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6">
       <c r="A118" s="2">
         <v>117</v>
       </c>
@@ -3489,8 +4554,14 @@
       <c r="D118" s="4">
         <v>638</v>
       </c>
-    </row>
-    <row r="119" spans="1:4">
+      <c r="E118" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F118" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6">
       <c r="A119" s="2">
         <v>118</v>
       </c>
@@ -3503,8 +4574,12 @@
       <c r="D119" s="4">
         <v>528</v>
       </c>
-    </row>
-    <row r="120" spans="1:4">
+      <c r="E119" s="4"/>
+      <c r="F119" s="4">
+        <v>764.12</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6">
       <c r="A120" s="2">
         <v>119</v>
       </c>
@@ -3517,8 +4592,14 @@
       <c r="D120" s="4">
         <v>249</v>
       </c>
-    </row>
-    <row r="121" spans="1:4">
+      <c r="E120" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F120" s="4">
+        <v>315.23</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6">
       <c r="A121" s="2">
         <v>120</v>
       </c>
@@ -3531,8 +4612,14 @@
       <c r="D121" s="4">
         <v>397</v>
       </c>
-    </row>
-    <row r="122" spans="1:4">
+      <c r="E121" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F121" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6">
       <c r="A122" s="2">
         <v>121</v>
       </c>
@@ -3545,8 +4632,12 @@
       <c r="D122" s="4">
         <v>698</v>
       </c>
-    </row>
-    <row r="123" spans="1:4">
+      <c r="E122" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F122" s="4"/>
+    </row>
+    <row r="123" spans="1:6">
       <c r="A123" s="2">
         <v>122</v>
       </c>
@@ -3559,8 +4650,14 @@
       <c r="D123" s="4">
         <v>598</v>
       </c>
-    </row>
-    <row r="124" spans="1:4">
+      <c r="E123" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F123" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6">
       <c r="A124" s="2">
         <v>123</v>
       </c>
@@ -3573,8 +4670,14 @@
       <c r="D124" s="4">
         <v>598</v>
       </c>
-    </row>
-    <row r="125" spans="1:4">
+      <c r="E124" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F124" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6">
       <c r="A125" s="2">
         <v>124</v>
       </c>
@@ -3587,8 +4690,14 @@
       <c r="D125" s="4">
         <v>755</v>
       </c>
-    </row>
-    <row r="126" spans="1:4">
+      <c r="E125" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F125" s="4">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6">
       <c r="A126" s="2">
         <v>125</v>
       </c>
@@ -3597,8 +4706,10 @@
       </c>
       <c r="C126" s="4"/>
       <c r="D126" s="4"/>
-    </row>
-    <row r="127" spans="1:4">
+      <c r="E126" s="4"/>
+      <c r="F126" s="4"/>
+    </row>
+    <row r="127" spans="1:6">
       <c r="A127" s="2">
         <v>126</v>
       </c>
@@ -3611,8 +4722,12 @@
       <c r="D127" s="4">
         <v>598</v>
       </c>
-    </row>
-    <row r="128" spans="1:4">
+      <c r="E127" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F127" s="4"/>
+    </row>
+    <row r="128" spans="1:6">
       <c r="A128" s="2">
         <v>127</v>
       </c>
@@ -3625,8 +4740,14 @@
       <c r="D128" s="4">
         <v>1999</v>
       </c>
-    </row>
-    <row r="129" spans="1:4">
+      <c r="E128" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F128" s="4">
+        <v>2599</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6">
       <c r="A129" s="2">
         <v>128</v>
       </c>
@@ -3635,8 +4756,10 @@
       </c>
       <c r="C129" s="4"/>
       <c r="D129" s="4"/>
-    </row>
-    <row r="130" spans="1:4">
+      <c r="E129" s="4"/>
+      <c r="F129" s="4"/>
+    </row>
+    <row r="130" spans="1:6">
       <c r="A130" s="2">
         <v>129</v>
       </c>
@@ -3649,8 +4772,14 @@
       <c r="D130" s="4">
         <v>598</v>
       </c>
-    </row>
-    <row r="131" spans="1:4">
+      <c r="E130" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F130" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6">
       <c r="A131" s="2">
         <v>130</v>
       </c>
@@ -3659,8 +4788,10 @@
       </c>
       <c r="C131" s="4"/>
       <c r="D131" s="4"/>
-    </row>
-    <row r="132" spans="1:4">
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
+    </row>
+    <row r="132" spans="1:6">
       <c r="A132" s="2">
         <v>131</v>
       </c>
@@ -3673,8 +4804,14 @@
       <c r="D132" s="4">
         <v>638</v>
       </c>
-    </row>
-    <row r="133" spans="1:4">
+      <c r="E132" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F132" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6">
       <c r="A133" s="2">
         <v>132</v>
       </c>
@@ -3687,8 +4824,14 @@
       <c r="D133" s="4">
         <v>145</v>
       </c>
-    </row>
-    <row r="134" spans="1:4">
+      <c r="E133" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F133" s="4">
+        <v>136.41</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6">
       <c r="A134" s="2">
         <v>133</v>
       </c>
@@ -3701,8 +4844,14 @@
       <c r="D134" s="4">
         <v>149</v>
       </c>
-    </row>
-    <row r="135" spans="1:4">
+      <c r="E134" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F134" s="4">
+        <v>287.5</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6">
       <c r="A135" s="2">
         <v>134</v>
       </c>
@@ -3711,8 +4860,14 @@
       </c>
       <c r="C135" s="4"/>
       <c r="D135" s="4"/>
-    </row>
-    <row r="136" spans="1:4">
+      <c r="E135" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F135" s="4">
+        <v>1334.54</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6">
       <c r="A136" s="2">
         <v>135</v>
       </c>
@@ -3725,8 +4880,14 @@
       <c r="D136" s="4">
         <v>1419</v>
       </c>
-    </row>
-    <row r="137" spans="1:4">
+      <c r="E136" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F136" s="4">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6">
       <c r="A137" s="2">
         <v>136</v>
       </c>
@@ -3739,8 +4900,14 @@
       <c r="D137" s="4">
         <v>185</v>
       </c>
-    </row>
-    <row r="138" spans="1:4">
+      <c r="E137" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F137" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6">
       <c r="A138" s="2">
         <v>137</v>
       </c>
@@ -3753,8 +4920,14 @@
       <c r="D138" s="4">
         <v>185</v>
       </c>
-    </row>
-    <row r="139" spans="1:4">
+      <c r="E138" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F138" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6">
       <c r="A139" s="2">
         <v>138</v>
       </c>
@@ -3767,8 +4940,14 @@
       <c r="D139" s="4">
         <v>185</v>
       </c>
-    </row>
-    <row r="140" spans="1:4">
+      <c r="E139" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F139" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6">
       <c r="A140" s="2">
         <v>139</v>
       </c>
@@ -3781,8 +4960,14 @@
       <c r="D140" s="4">
         <v>718</v>
       </c>
-    </row>
-    <row r="141" spans="1:4">
+      <c r="E140" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F140" s="4">
+        <v>730.77</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6">
       <c r="A141" s="2">
         <v>140</v>
       </c>
@@ -3795,8 +4980,14 @@
       <c r="D141" s="4">
         <v>639</v>
       </c>
-    </row>
-    <row r="142" spans="1:4">
+      <c r="E141" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F141" s="4">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6">
       <c r="A142" s="2">
         <v>141</v>
       </c>
@@ -3805,8 +4996,10 @@
       </c>
       <c r="C142" s="4"/>
       <c r="D142" s="4"/>
-    </row>
-    <row r="143" spans="1:4">
+      <c r="E142" s="4"/>
+      <c r="F142" s="4"/>
+    </row>
+    <row r="143" spans="1:6">
       <c r="A143" s="2">
         <v>142</v>
       </c>
@@ -3819,8 +5012,14 @@
       <c r="D143" s="4">
         <v>70</v>
       </c>
-    </row>
-    <row r="144" spans="1:4">
+      <c r="E143" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F143" s="4">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6">
       <c r="A144" s="2">
         <v>143</v>
       </c>
@@ -3833,8 +5032,14 @@
       <c r="D144" s="4">
         <v>70</v>
       </c>
-    </row>
-    <row r="145" spans="1:4">
+      <c r="E144" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F144" s="4">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6">
       <c r="A145" s="2">
         <v>144</v>
       </c>
@@ -3847,8 +5052,14 @@
       <c r="D145" s="4">
         <v>4998</v>
       </c>
-    </row>
-    <row r="146" spans="1:4">
+      <c r="E145" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F145" s="4">
+        <v>6650.99</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6">
       <c r="A146" s="2">
         <v>145</v>
       </c>
@@ -3861,8 +5072,14 @@
       <c r="D146" s="4">
         <v>597</v>
       </c>
-    </row>
-    <row r="147" spans="1:4">
+      <c r="E146" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="F146" s="4">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6">
       <c r="A147" s="2">
         <v>146</v>
       </c>
@@ -3871,8 +5088,14 @@
       </c>
       <c r="C147" s="4"/>
       <c r="D147" s="4"/>
-    </row>
-    <row r="148" spans="1:4">
+      <c r="E147" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F147" s="4">
+        <v>2690</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6">
       <c r="A148" s="2">
         <v>147</v>
       </c>
@@ -3881,8 +5104,10 @@
       </c>
       <c r="C148" s="4"/>
       <c r="D148" s="4"/>
-    </row>
-    <row r="149" spans="1:4">
+      <c r="E148" s="4"/>
+      <c r="F148" s="4"/>
+    </row>
+    <row r="149" spans="1:6">
       <c r="A149" s="2">
         <v>148</v>
       </c>
@@ -3895,8 +5120,14 @@
       <c r="D149" s="4">
         <v>639</v>
       </c>
-    </row>
-    <row r="150" spans="1:4">
+      <c r="E149" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F149" s="4">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6">
       <c r="A150" s="2">
         <v>149</v>
       </c>
@@ -3909,8 +5140,14 @@
       <c r="D150" s="4">
         <v>788</v>
       </c>
-    </row>
-    <row r="151" spans="1:4">
+      <c r="E150" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F150" s="4">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6">
       <c r="A151" s="2">
         <v>150</v>
       </c>
@@ -3923,8 +5160,14 @@
       <c r="D151" s="4">
         <v>788</v>
       </c>
-    </row>
-    <row r="152" spans="1:4">
+      <c r="E151" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F151" s="4">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6">
       <c r="A152" s="2">
         <v>151</v>
       </c>
@@ -3937,8 +5180,14 @@
       <c r="D152" s="4">
         <v>188</v>
       </c>
-    </row>
-    <row r="153" spans="1:4">
+      <c r="E152" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F152" s="4">
+        <v>243.33</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6">
       <c r="A153" s="2">
         <v>152</v>
       </c>
@@ -3951,8 +5200,10 @@
       <c r="D153" s="4">
         <v>488</v>
       </c>
-    </row>
-    <row r="154" spans="1:4">
+      <c r="E153" s="4"/>
+      <c r="F153" s="4"/>
+    </row>
+    <row r="154" spans="1:6">
       <c r="A154" s="2">
         <v>153</v>
       </c>
@@ -3965,8 +5216,14 @@
       <c r="D154" s="4">
         <v>788</v>
       </c>
-    </row>
-    <row r="155" spans="1:4">
+      <c r="E154" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F154" s="4">
+        <v>824.86</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6">
       <c r="A155" s="2">
         <v>154</v>
       </c>
@@ -3979,8 +5236,14 @@
       <c r="D155" s="4">
         <v>788</v>
       </c>
-    </row>
-    <row r="156" spans="1:4">
+      <c r="E155" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F155" s="4">
+        <v>824.86</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6">
       <c r="A156" s="2">
         <v>155</v>
       </c>
@@ -3993,8 +5256,14 @@
       <c r="D156" s="4">
         <v>119</v>
       </c>
-    </row>
-    <row r="157" spans="1:4">
+      <c r="E156" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F156" s="4">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6">
       <c r="A157" s="2">
         <v>156</v>
       </c>
@@ -4007,8 +5276,14 @@
       <c r="D157" s="4">
         <v>283</v>
       </c>
-    </row>
-    <row r="158" spans="1:4">
+      <c r="E157" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F157" s="4">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6">
       <c r="A158" s="2">
         <v>157</v>
       </c>
@@ -4017,8 +5292,10 @@
       </c>
       <c r="C158" s="4"/>
       <c r="D158" s="4"/>
-    </row>
-    <row r="159" spans="1:4">
+      <c r="E158" s="4"/>
+      <c r="F158" s="4"/>
+    </row>
+    <row r="159" spans="1:6">
       <c r="A159" s="2">
         <v>158</v>
       </c>
@@ -4027,8 +5304,14 @@
       </c>
       <c r="C159" s="4"/>
       <c r="D159" s="4"/>
-    </row>
-    <row r="160" spans="1:4">
+      <c r="E159" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F159" s="4">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6">
       <c r="A160" s="2">
         <v>159</v>
       </c>
@@ -4041,8 +5324,14 @@
       <c r="D160" s="4">
         <v>849</v>
       </c>
-    </row>
-    <row r="161" spans="1:4">
+      <c r="E160" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F160" s="4">
+        <v>1697</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6">
       <c r="A161" s="2">
         <v>160</v>
       </c>
@@ -4055,8 +5344,14 @@
       <c r="D161" s="4">
         <v>699</v>
       </c>
-    </row>
-    <row r="162" spans="1:4">
+      <c r="E161" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F161" s="4">
+        <v>730.77</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6">
       <c r="A162" s="2">
         <v>161</v>
       </c>
@@ -4069,8 +5364,14 @@
       <c r="D162" s="4">
         <v>679</v>
       </c>
-    </row>
-    <row r="163" spans="1:4">
+      <c r="E162" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="F162" s="4">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6">
       <c r="A163" s="2">
         <v>162</v>
       </c>
@@ -4083,8 +5384,14 @@
       <c r="D163" s="4">
         <v>689</v>
       </c>
-    </row>
-    <row r="164" spans="1:4">
+      <c r="E163" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F163" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6">
       <c r="A164" s="2">
         <v>163</v>
       </c>
@@ -4097,8 +5404,14 @@
       <c r="D164" s="4">
         <v>689</v>
       </c>
-    </row>
-    <row r="165" spans="1:4">
+      <c r="E164" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F164" s="4">
+        <v>720.32</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6">
       <c r="A165" s="2">
         <v>164</v>
       </c>
@@ -4111,8 +5424,14 @@
       <c r="D165" s="4">
         <v>158</v>
       </c>
-    </row>
-    <row r="166" spans="1:4">
+      <c r="E165" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F165" s="4">
+        <v>303.26</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6">
       <c r="A166" s="2">
         <v>165</v>
       </c>
@@ -4121,8 +5440,14 @@
       </c>
       <c r="C166" s="4"/>
       <c r="D166" s="4"/>
-    </row>
-    <row r="167" spans="1:4">
+      <c r="E166" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F166" s="4">
+        <v>2549</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6">
       <c r="A167" s="2">
         <v>166</v>
       </c>
@@ -4135,142 +5460,174 @@
       <c r="D167" s="4">
         <v>1199</v>
       </c>
+      <c r="E167" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F167" s="4">
+        <v>1433.91</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1">
-    <cfRule type="duplicateValues" dxfId="66" priority="65"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="66"/>
-    <cfRule type="duplicateValues" dxfId="64" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B134">
-    <cfRule type="duplicateValues" dxfId="63" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B3">
-    <cfRule type="duplicateValues" dxfId="62" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="76"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B13">
-    <cfRule type="duplicateValues" dxfId="61" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="74"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B35">
-    <cfRule type="duplicateValues" dxfId="60" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4">
-    <cfRule type="duplicateValues" dxfId="59" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="75"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:B6">
-    <cfRule type="duplicateValues" dxfId="58" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:B10">
-    <cfRule type="duplicateValues" dxfId="57" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="78"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:B13">
-    <cfRule type="duplicateValues" dxfId="56" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:B35">
-    <cfRule type="duplicateValues" dxfId="55" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B36:B55">
-    <cfRule type="duplicateValues" dxfId="54" priority="55"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B56">
-    <cfRule type="duplicateValues" dxfId="52" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B57:B58">
-    <cfRule type="duplicateValues" dxfId="51" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59:B60">
-    <cfRule type="duplicateValues" dxfId="50" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B61">
-    <cfRule type="duplicateValues" dxfId="49" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B62:B90">
-    <cfRule type="duplicateValues" dxfId="48" priority="48"/>
-    <cfRule type="duplicateValues" dxfId="47" priority="49"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B91:B92">
-    <cfRule type="duplicateValues" dxfId="45" priority="41"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="42"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="43"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="58"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93:B94">
-    <cfRule type="duplicateValues" dxfId="41" priority="39"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95:B134">
-    <cfRule type="duplicateValues" dxfId="39" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="37"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B135:B164">
-    <cfRule type="duplicateValues" dxfId="36" priority="33"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B165">
-    <cfRule type="duplicateValues" dxfId="34" priority="29"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="31"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="46"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B90">
-    <cfRule type="duplicateValues" dxfId="30" priority="45"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="46"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="61"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="27" priority="26"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="27"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="23" priority="23"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="24"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="20" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="17" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="16" priority="16"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="17"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="13" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="10" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="9" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1">
+    <cfRule type="duplicateValues" dxfId="19" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1">
+    <cfRule type="duplicateValues" dxfId="16" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1">
+    <cfRule type="duplicateValues" dxfId="15" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1">
+    <cfRule type="duplicateValues" dxfId="12" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1">
+    <cfRule type="duplicateValues" dxfId="9" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1">
+    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto backup 2026-07-01 04:05:02
</commit_message>
<xml_diff>
--- a/SwissTechShehzad/27-06-2026/27-06-2026.xlsx
+++ b/SwissTechShehzad/27-06-2026/27-06-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\27-06-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58FEAB30-7628-4AD3-AAC3-F4B2BA5BEEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF126D03-354F-44B0-9CEC-16E331D6D3BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1905" windowWidth="29040" windowHeight="17520" xr2:uid="{8BCFAE85-CB20-435D-AEB6-6494F3D318DE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="211">
   <si>
     <t>Sr No</t>
   </si>
@@ -667,6 +667,9 @@
   </si>
   <si>
     <t>newegg.com</t>
+  </si>
+  <si>
+    <t>1.090.99</t>
   </si>
 </sst>
 </file>
@@ -780,167 +783,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="101">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="85">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -4446,6 +4289,12 @@
       <c r="F93" s="4">
         <v>529</v>
       </c>
+      <c r="G93" t="s">
+        <v>208</v>
+      </c>
+      <c r="H93">
+        <v>319</v>
+      </c>
     </row>
     <row r="94" spans="1:8">
       <c r="A94" s="2">
@@ -4466,6 +4315,12 @@
       <c r="F94" s="4">
         <v>175</v>
       </c>
+      <c r="G94" t="s">
+        <v>207</v>
+      </c>
+      <c r="H94">
+        <v>159.94999999999999</v>
+      </c>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" s="2">
@@ -4486,6 +4341,12 @@
       <c r="F95" s="4">
         <v>175</v>
       </c>
+      <c r="G95" t="s">
+        <v>207</v>
+      </c>
+      <c r="H95">
+        <v>159.65</v>
+      </c>
     </row>
     <row r="96" spans="1:8">
       <c r="A96" s="2">
@@ -4506,8 +4367,14 @@
       <c r="F96" s="4">
         <v>137.33000000000001</v>
       </c>
-    </row>
-    <row r="97" spans="1:6">
+      <c r="G96" t="s">
+        <v>208</v>
+      </c>
+      <c r="H96">
+        <v>104.99</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -4526,8 +4393,14 @@
       <c r="F97" s="4">
         <v>675</v>
       </c>
-    </row>
-    <row r="98" spans="1:6">
+      <c r="G97" t="s">
+        <v>208</v>
+      </c>
+      <c r="H97">
+        <v>351.45</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -4542,8 +4415,14 @@
       <c r="F98" s="4">
         <v>1289.51</v>
       </c>
-    </row>
-    <row r="99" spans="1:6">
+      <c r="G98" t="s">
+        <v>209</v>
+      </c>
+      <c r="H98" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -4554,8 +4433,14 @@
       <c r="D99" s="4"/>
       <c r="E99" s="4"/>
       <c r="F99" s="4"/>
-    </row>
-    <row r="100" spans="1:6">
+      <c r="G99" t="s">
+        <v>207</v>
+      </c>
+      <c r="H99">
+        <v>696.49</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -4574,8 +4459,14 @@
       <c r="F100" s="4">
         <v>315.23</v>
       </c>
-    </row>
-    <row r="101" spans="1:6">
+      <c r="G100" t="s">
+        <v>208</v>
+      </c>
+      <c r="H100">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -4590,8 +4481,14 @@
       <c r="F101" s="4">
         <v>2914.2</v>
       </c>
-    </row>
-    <row r="102" spans="1:6">
+      <c r="G101" t="s">
+        <v>209</v>
+      </c>
+      <c r="H101">
+        <v>2379</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -4606,8 +4503,14 @@
       <c r="F102" s="4">
         <v>1928.14</v>
       </c>
-    </row>
-    <row r="103" spans="1:6">
+      <c r="G102" t="s">
+        <v>208</v>
+      </c>
+      <c r="H102">
+        <v>682.02</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -4626,8 +4529,14 @@
       <c r="F103" s="4">
         <v>1347.98</v>
       </c>
-    </row>
-    <row r="104" spans="1:6">
+      <c r="G103" t="s">
+        <v>207</v>
+      </c>
+      <c r="H103">
+        <v>1099.95</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -4642,8 +4551,14 @@
       <c r="F104" s="4">
         <v>1169.69</v>
       </c>
-    </row>
-    <row r="105" spans="1:6">
+      <c r="G104" t="s">
+        <v>207</v>
+      </c>
+      <c r="H104">
+        <v>666.99</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -4658,8 +4573,14 @@
       <c r="F105" s="4">
         <v>2748.99</v>
       </c>
-    </row>
-    <row r="106" spans="1:6">
+      <c r="G105" t="s">
+        <v>207</v>
+      </c>
+      <c r="H105">
+        <v>1037.99</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -4678,8 +4599,14 @@
       <c r="F106" s="4">
         <v>855</v>
       </c>
-    </row>
-    <row r="107" spans="1:6">
+      <c r="G106" t="s">
+        <v>208</v>
+      </c>
+      <c r="H106">
+        <v>429.95</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -4699,7 +4626,7 @@
         <v>720.32</v>
       </c>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" spans="1:8">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -4718,8 +4645,14 @@
       <c r="F108" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="109" spans="1:6">
+      <c r="G108" t="s">
+        <v>207</v>
+      </c>
+      <c r="H108">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -4731,7 +4664,7 @@
       <c r="E109" s="4"/>
       <c r="F109" s="4"/>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" spans="1:8">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -4744,8 +4677,14 @@
       <c r="F110" s="4">
         <v>1436.35</v>
       </c>
-    </row>
-    <row r="111" spans="1:6">
+      <c r="G110" t="s">
+        <v>208</v>
+      </c>
+      <c r="H110">
+        <v>747.35</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -4765,7 +4704,7 @@
         <v>40.54</v>
       </c>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" spans="1:8">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -4784,8 +4723,14 @@
       <c r="F112" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="113" spans="1:6">
+      <c r="G112" t="s">
+        <v>208</v>
+      </c>
+      <c r="H112">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -4804,8 +4749,14 @@
       <c r="F113" s="4">
         <v>315.23</v>
       </c>
-    </row>
-    <row r="114" spans="1:6">
+      <c r="G113" t="s">
+        <v>208</v>
+      </c>
+      <c r="H113">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -4816,8 +4767,11 @@
       <c r="D114" s="4"/>
       <c r="E114" s="4"/>
       <c r="F114" s="4"/>
-    </row>
-    <row r="115" spans="1:6">
+      <c r="H114">
+        <v>1165.99</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8">
       <c r="A115" s="2">
         <v>114</v>
       </c>
@@ -4833,7 +4787,7 @@
       <c r="E115" s="4"/>
       <c r="F115" s="4"/>
     </row>
-    <row r="116" spans="1:6">
+    <row r="116" spans="1:8">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -4852,8 +4806,14 @@
       <c r="F116" s="4">
         <v>616.64</v>
       </c>
-    </row>
-    <row r="117" spans="1:6">
+      <c r="G116" t="s">
+        <v>208</v>
+      </c>
+      <c r="H116">
+        <v>631.04</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -4872,8 +4832,14 @@
       <c r="F117" s="4">
         <v>782.56</v>
       </c>
-    </row>
-    <row r="118" spans="1:6">
+      <c r="G117" t="s">
+        <v>209</v>
+      </c>
+      <c r="H117">
+        <v>399.99</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8">
       <c r="A118" s="2">
         <v>117</v>
       </c>
@@ -4892,8 +4858,14 @@
       <c r="F118" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="119" spans="1:6">
+      <c r="G118" t="s">
+        <v>207</v>
+      </c>
+      <c r="H118">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8">
       <c r="A119" s="2">
         <v>118</v>
       </c>
@@ -4910,8 +4882,14 @@
       <c r="F119" s="4">
         <v>764.12</v>
       </c>
-    </row>
-    <row r="120" spans="1:6">
+      <c r="G119" t="s">
+        <v>207</v>
+      </c>
+      <c r="H119">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8">
       <c r="A120" s="2">
         <v>119</v>
       </c>
@@ -4930,8 +4908,14 @@
       <c r="F120" s="4">
         <v>315.23</v>
       </c>
-    </row>
-    <row r="121" spans="1:6">
+      <c r="G120" t="s">
+        <v>208</v>
+      </c>
+      <c r="H120">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8">
       <c r="A121" s="2">
         <v>120</v>
       </c>
@@ -4950,8 +4934,14 @@
       <c r="F121" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="122" spans="1:6">
+      <c r="G121" t="s">
+        <v>207</v>
+      </c>
+      <c r="H121">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8">
       <c r="A122" s="2">
         <v>121</v>
       </c>
@@ -4968,8 +4958,14 @@
         <v>196</v>
       </c>
       <c r="F122" s="4"/>
-    </row>
-    <row r="123" spans="1:6">
+      <c r="G122" t="s">
+        <v>207</v>
+      </c>
+      <c r="H122">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8">
       <c r="A123" s="2">
         <v>122</v>
       </c>
@@ -4988,8 +4984,14 @@
       <c r="F123" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="124" spans="1:6">
+      <c r="G123" t="s">
+        <v>207</v>
+      </c>
+      <c r="H123">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8">
       <c r="A124" s="2">
         <v>123</v>
       </c>
@@ -5008,8 +5010,14 @@
       <c r="F124" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="125" spans="1:6">
+      <c r="G124" t="s">
+        <v>207</v>
+      </c>
+      <c r="H124">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8">
       <c r="A125" s="2">
         <v>124</v>
       </c>
@@ -5028,8 +5036,14 @@
       <c r="F125" s="4">
         <v>849</v>
       </c>
-    </row>
-    <row r="126" spans="1:6">
+      <c r="G125" t="s">
+        <v>208</v>
+      </c>
+      <c r="H125">
+        <v>577.91</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8">
       <c r="A126" s="2">
         <v>125</v>
       </c>
@@ -5040,8 +5054,14 @@
       <c r="D126" s="4"/>
       <c r="E126" s="4"/>
       <c r="F126" s="4"/>
-    </row>
-    <row r="127" spans="1:6">
+      <c r="G126" t="s">
+        <v>208</v>
+      </c>
+      <c r="H126">
+        <v>711.61</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8">
       <c r="A127" s="2">
         <v>126</v>
       </c>
@@ -5058,8 +5078,14 @@
         <v>196</v>
       </c>
       <c r="F127" s="4"/>
-    </row>
-    <row r="128" spans="1:6">
+      <c r="G127" t="s">
+        <v>207</v>
+      </c>
+      <c r="H127">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8">
       <c r="A128" s="2">
         <v>127</v>
       </c>
@@ -5079,7 +5105,7 @@
         <v>2599</v>
       </c>
     </row>
-    <row r="129" spans="1:6">
+    <row r="129" spans="1:8">
       <c r="A129" s="2">
         <v>128</v>
       </c>
@@ -5091,7 +5117,7 @@
       <c r="E129" s="4"/>
       <c r="F129" s="4"/>
     </row>
-    <row r="130" spans="1:6">
+    <row r="130" spans="1:8">
       <c r="A130" s="2">
         <v>129</v>
       </c>
@@ -5110,8 +5136,14 @@
       <c r="F130" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="131" spans="1:6">
+      <c r="G130" t="s">
+        <v>207</v>
+      </c>
+      <c r="H130">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8">
       <c r="A131" s="2">
         <v>130</v>
       </c>
@@ -5123,7 +5155,7 @@
       <c r="E131" s="4"/>
       <c r="F131" s="4"/>
     </row>
-    <row r="132" spans="1:6">
+    <row r="132" spans="1:8">
       <c r="A132" s="2">
         <v>131</v>
       </c>
@@ -5142,8 +5174,14 @@
       <c r="F132" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="133" spans="1:6">
+      <c r="G132" t="s">
+        <v>207</v>
+      </c>
+      <c r="H132">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8">
       <c r="A133" s="2">
         <v>132</v>
       </c>
@@ -5162,8 +5200,14 @@
       <c r="F133" s="4">
         <v>136.41</v>
       </c>
-    </row>
-    <row r="134" spans="1:6">
+      <c r="G133" t="s">
+        <v>207</v>
+      </c>
+      <c r="H133">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8">
       <c r="A134" s="2">
         <v>133</v>
       </c>
@@ -5182,8 +5226,14 @@
       <c r="F134" s="4">
         <v>287.5</v>
       </c>
-    </row>
-    <row r="135" spans="1:6">
+      <c r="G134" t="s">
+        <v>208</v>
+      </c>
+      <c r="H134">
+        <v>84.99</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8">
       <c r="A135" s="2">
         <v>134</v>
       </c>
@@ -5198,8 +5248,14 @@
       <c r="F135" s="4">
         <v>1334.54</v>
       </c>
-    </row>
-    <row r="136" spans="1:6">
+      <c r="G135" t="s">
+        <v>207</v>
+      </c>
+      <c r="H135">
+        <v>789.99</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8">
       <c r="A136" s="2">
         <v>135</v>
       </c>
@@ -5219,7 +5275,7 @@
         <v>1950</v>
       </c>
     </row>
-    <row r="137" spans="1:6">
+    <row r="137" spans="1:8">
       <c r="A137" s="2">
         <v>136</v>
       </c>
@@ -5238,8 +5294,14 @@
       <c r="F137" s="4">
         <v>175</v>
       </c>
-    </row>
-    <row r="138" spans="1:6">
+      <c r="G137" t="s">
+        <v>207</v>
+      </c>
+      <c r="H137">
+        <v>159.94999999999999</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8">
       <c r="A138" s="2">
         <v>137</v>
       </c>
@@ -5258,8 +5320,14 @@
       <c r="F138" s="4">
         <v>175</v>
       </c>
-    </row>
-    <row r="139" spans="1:6">
+      <c r="G138" t="s">
+        <v>207</v>
+      </c>
+      <c r="H138">
+        <v>159.94999999999999</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8">
       <c r="A139" s="2">
         <v>138</v>
       </c>
@@ -5278,8 +5346,14 @@
       <c r="F139" s="4">
         <v>175</v>
       </c>
-    </row>
-    <row r="140" spans="1:6">
+      <c r="G139" t="s">
+        <v>207</v>
+      </c>
+      <c r="H139">
+        <v>159.94999999999999</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8">
       <c r="A140" s="2">
         <v>139</v>
       </c>
@@ -5298,8 +5372,14 @@
       <c r="F140" s="4">
         <v>730.77</v>
       </c>
-    </row>
-    <row r="141" spans="1:6">
+      <c r="G140" t="s">
+        <v>208</v>
+      </c>
+      <c r="H140">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8">
       <c r="A141" s="2">
         <v>140</v>
       </c>
@@ -5318,8 +5398,14 @@
       <c r="F141" s="4">
         <v>745</v>
       </c>
-    </row>
-    <row r="142" spans="1:6">
+      <c r="G141" t="s">
+        <v>208</v>
+      </c>
+      <c r="H141">
+        <v>549.95000000000005</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8">
       <c r="A142" s="2">
         <v>141</v>
       </c>
@@ -5331,7 +5417,7 @@
       <c r="E142" s="4"/>
       <c r="F142" s="4"/>
     </row>
-    <row r="143" spans="1:6">
+    <row r="143" spans="1:8">
       <c r="A143" s="2">
         <v>142</v>
       </c>
@@ -5350,8 +5436,14 @@
       <c r="F143" s="4">
         <v>95</v>
       </c>
-    </row>
-    <row r="144" spans="1:6">
+      <c r="G143" t="s">
+        <v>207</v>
+      </c>
+      <c r="H143">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8">
       <c r="A144" s="2">
         <v>143</v>
       </c>
@@ -5370,8 +5462,14 @@
       <c r="F144" s="4">
         <v>95</v>
       </c>
-    </row>
-    <row r="145" spans="1:6">
+      <c r="G144" t="s">
+        <v>207</v>
+      </c>
+      <c r="H144">
+        <v>79.95</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8">
       <c r="A145" s="2">
         <v>144</v>
       </c>
@@ -5390,8 +5488,14 @@
       <c r="F145" s="4">
         <v>6650.99</v>
       </c>
-    </row>
-    <row r="146" spans="1:6">
+      <c r="G145" t="s">
+        <v>208</v>
+      </c>
+      <c r="H145">
+        <v>3899</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8">
       <c r="A146" s="2">
         <v>145</v>
       </c>
@@ -5410,8 +5514,14 @@
       <c r="F146" s="4">
         <v>699</v>
       </c>
-    </row>
-    <row r="147" spans="1:6">
+      <c r="G146" t="s">
+        <v>208</v>
+      </c>
+      <c r="H146">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8">
       <c r="A147" s="2">
         <v>146</v>
       </c>
@@ -5426,8 +5536,14 @@
       <c r="F147" s="4">
         <v>2690</v>
       </c>
-    </row>
-    <row r="148" spans="1:6">
+      <c r="G147" t="s">
+        <v>208</v>
+      </c>
+      <c r="H147">
+        <v>1249.99</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8">
       <c r="A148" s="2">
         <v>147</v>
       </c>
@@ -5438,8 +5554,14 @@
       <c r="D148" s="4"/>
       <c r="E148" s="4"/>
       <c r="F148" s="4"/>
-    </row>
-    <row r="149" spans="1:6">
+      <c r="G148" t="s">
+        <v>208</v>
+      </c>
+      <c r="H148">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8">
       <c r="A149" s="2">
         <v>148</v>
       </c>
@@ -5458,8 +5580,14 @@
       <c r="F149" s="4">
         <v>745</v>
       </c>
-    </row>
-    <row r="150" spans="1:6">
+      <c r="G149" t="s">
+        <v>208</v>
+      </c>
+      <c r="H149">
+        <v>549.95000000000005</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8">
       <c r="A150" s="2">
         <v>149</v>
       </c>
@@ -5478,8 +5606,14 @@
       <c r="F150" s="4">
         <v>788</v>
       </c>
-    </row>
-    <row r="151" spans="1:6">
+      <c r="G150" t="s">
+        <v>207</v>
+      </c>
+      <c r="H150">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8">
       <c r="A151" s="2">
         <v>150</v>
       </c>
@@ -5498,8 +5632,14 @@
       <c r="F151" s="4">
         <v>788</v>
       </c>
-    </row>
-    <row r="152" spans="1:6">
+      <c r="G151" t="s">
+        <v>207</v>
+      </c>
+      <c r="H151">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8">
       <c r="A152" s="2">
         <v>151</v>
       </c>
@@ -5518,8 +5658,14 @@
       <c r="F152" s="4">
         <v>243.33</v>
       </c>
-    </row>
-    <row r="153" spans="1:6">
+      <c r="G152" t="s">
+        <v>207</v>
+      </c>
+      <c r="H152">
+        <v>129.99</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8">
       <c r="A153" s="2">
         <v>152</v>
       </c>
@@ -5534,8 +5680,14 @@
       </c>
       <c r="E153" s="4"/>
       <c r="F153" s="4"/>
-    </row>
-    <row r="154" spans="1:6">
+      <c r="G153" t="s">
+        <v>208</v>
+      </c>
+      <c r="H153">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8">
       <c r="A154" s="2">
         <v>153</v>
       </c>
@@ -5554,8 +5706,14 @@
       <c r="F154" s="4">
         <v>824.86</v>
       </c>
-    </row>
-    <row r="155" spans="1:6">
+      <c r="G154" t="s">
+        <v>207</v>
+      </c>
+      <c r="H154">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8">
       <c r="A155" s="2">
         <v>154</v>
       </c>
@@ -5574,8 +5732,14 @@
       <c r="F155" s="4">
         <v>824.86</v>
       </c>
-    </row>
-    <row r="156" spans="1:6">
+      <c r="G155" t="s">
+        <v>207</v>
+      </c>
+      <c r="H155">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8">
       <c r="A156" s="2">
         <v>155</v>
       </c>
@@ -5594,8 +5758,14 @@
       <c r="F156" s="4">
         <v>129</v>
       </c>
-    </row>
-    <row r="157" spans="1:6">
+      <c r="G156" t="s">
+        <v>208</v>
+      </c>
+      <c r="H156">
+        <v>91.99</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8">
       <c r="A157" s="2">
         <v>156</v>
       </c>
@@ -5614,8 +5784,14 @@
       <c r="F157" s="4">
         <v>398</v>
       </c>
-    </row>
-    <row r="158" spans="1:6">
+      <c r="G157" t="s">
+        <v>208</v>
+      </c>
+      <c r="H157">
+        <v>379.95</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8">
       <c r="A158" s="2">
         <v>157</v>
       </c>
@@ -5626,8 +5802,14 @@
       <c r="D158" s="4"/>
       <c r="E158" s="4"/>
       <c r="F158" s="4"/>
-    </row>
-    <row r="159" spans="1:6">
+      <c r="G158" t="s">
+        <v>207</v>
+      </c>
+      <c r="H158">
+        <v>1449.99</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8">
       <c r="A159" s="2">
         <v>158</v>
       </c>
@@ -5642,8 +5824,14 @@
       <c r="F159" s="4">
         <v>988</v>
       </c>
-    </row>
-    <row r="160" spans="1:6">
+      <c r="G159" t="s">
+        <v>208</v>
+      </c>
+      <c r="H159">
+        <v>879.95</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8">
       <c r="A160" s="2">
         <v>159</v>
       </c>
@@ -5662,8 +5850,14 @@
       <c r="F160" s="4">
         <v>1697</v>
       </c>
-    </row>
-    <row r="161" spans="1:6">
+      <c r="G160" t="s">
+        <v>208</v>
+      </c>
+      <c r="H160">
+        <v>1399.95</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8">
       <c r="A161" s="2">
         <v>160</v>
       </c>
@@ -5682,8 +5876,14 @@
       <c r="F161" s="4">
         <v>730.77</v>
       </c>
-    </row>
-    <row r="162" spans="1:6">
+      <c r="G161" t="s">
+        <v>207</v>
+      </c>
+      <c r="H161">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8">
       <c r="A162" s="2">
         <v>161</v>
       </c>
@@ -5702,8 +5902,14 @@
       <c r="F162" s="4">
         <v>699</v>
       </c>
-    </row>
-    <row r="163" spans="1:6">
+      <c r="G162" t="s">
+        <v>208</v>
+      </c>
+      <c r="H162">
+        <v>448.88</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8">
       <c r="A163" s="2">
         <v>162</v>
       </c>
@@ -5722,8 +5928,14 @@
       <c r="F163" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="164" spans="1:6">
+      <c r="G163" t="s">
+        <v>207</v>
+      </c>
+      <c r="H163">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8">
       <c r="A164" s="2">
         <v>163</v>
       </c>
@@ -5742,8 +5954,14 @@
       <c r="F164" s="4">
         <v>720.32</v>
       </c>
-    </row>
-    <row r="165" spans="1:6">
+      <c r="G164" t="s">
+        <v>207</v>
+      </c>
+      <c r="H164">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8">
       <c r="A165" s="2">
         <v>164</v>
       </c>
@@ -5763,7 +5981,7 @@
         <v>303.26</v>
       </c>
     </row>
-    <row r="166" spans="1:6">
+    <row r="166" spans="1:8">
       <c r="A166" s="2">
         <v>165</v>
       </c>
@@ -5779,7 +5997,7 @@
         <v>2549</v>
       </c>
     </row>
-    <row r="167" spans="1:6">
+    <row r="167" spans="1:8">
       <c r="A167" s="2">
         <v>166</v>
       </c>
@@ -5798,168 +6016,174 @@
       <c r="F167" s="4">
         <v>1433.91</v>
       </c>
+      <c r="G167" t="s">
+        <v>208</v>
+      </c>
+      <c r="H167">
+        <v>900.51</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1">
-    <cfRule type="duplicateValues" dxfId="100" priority="79"/>
-    <cfRule type="duplicateValues" dxfId="99" priority="80"/>
-    <cfRule type="duplicateValues" dxfId="98" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B134">
-    <cfRule type="duplicateValues" dxfId="97" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B3">
-    <cfRule type="duplicateValues" dxfId="96" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="76"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B13">
-    <cfRule type="duplicateValues" dxfId="95" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="74"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B35">
-    <cfRule type="duplicateValues" dxfId="94" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4">
-    <cfRule type="duplicateValues" dxfId="93" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="75"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:B6">
-    <cfRule type="duplicateValues" dxfId="92" priority="77"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:B10">
-    <cfRule type="duplicateValues" dxfId="91" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="78"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:B13">
-    <cfRule type="duplicateValues" dxfId="90" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:B35">
-    <cfRule type="duplicateValues" dxfId="89" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B36:B55">
-    <cfRule type="duplicateValues" dxfId="88" priority="69"/>
-    <cfRule type="duplicateValues" dxfId="87" priority="70"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B56">
-    <cfRule type="duplicateValues" dxfId="86" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B57:B58">
-    <cfRule type="duplicateValues" dxfId="85" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59:B60">
-    <cfRule type="duplicateValues" dxfId="84" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B61">
-    <cfRule type="duplicateValues" dxfId="83" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B62:B90">
-    <cfRule type="duplicateValues" dxfId="82" priority="62"/>
-    <cfRule type="duplicateValues" dxfId="81" priority="63"/>
-    <cfRule type="duplicateValues" dxfId="80" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B91:B92">
-    <cfRule type="duplicateValues" dxfId="79" priority="55"/>
-    <cfRule type="duplicateValues" dxfId="78" priority="56"/>
-    <cfRule type="duplicateValues" dxfId="77" priority="57"/>
-    <cfRule type="duplicateValues" dxfId="76" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="58"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93:B94">
-    <cfRule type="duplicateValues" dxfId="75" priority="53"/>
-    <cfRule type="duplicateValues" dxfId="74" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95:B134">
-    <cfRule type="duplicateValues" dxfId="73" priority="50"/>
-    <cfRule type="duplicateValues" dxfId="72" priority="51"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B135:B164">
-    <cfRule type="duplicateValues" dxfId="70" priority="47"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B165">
-    <cfRule type="duplicateValues" dxfId="68" priority="43"/>
-    <cfRule type="duplicateValues" dxfId="67" priority="44"/>
-    <cfRule type="duplicateValues" dxfId="66" priority="45"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="46"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B90">
-    <cfRule type="duplicateValues" dxfId="64" priority="59"/>
-    <cfRule type="duplicateValues" dxfId="63" priority="60"/>
-    <cfRule type="duplicateValues" dxfId="62" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="61"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="61" priority="40"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="41"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="58" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="57" priority="37"/>
-    <cfRule type="duplicateValues" dxfId="56" priority="38"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="54" priority="33"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="34"/>
-    <cfRule type="duplicateValues" dxfId="52" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="51" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="50" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="31"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="47" priority="26"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="27"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="44" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="43" priority="23"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="24"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="duplicateValues" dxfId="40" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="duplicateValues" dxfId="37" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="duplicateValues" dxfId="36" priority="16"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="17"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1">
-    <cfRule type="duplicateValues" dxfId="27" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1">
-    <cfRule type="duplicateValues" dxfId="24" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1">
-    <cfRule type="duplicateValues" dxfId="23" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1">
-    <cfRule type="duplicateValues" dxfId="20" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1">
-    <cfRule type="duplicateValues" dxfId="17" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1">
-    <cfRule type="duplicateValues" dxfId="16" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto backup 2026-07-01 08:35:02
</commit_message>
<xml_diff>
--- a/SwissTechShehzad/27-06-2026/27-06-2026.xlsx
+++ b/SwissTechShehzad/27-06-2026/27-06-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\27-06-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF126D03-354F-44B0-9CEC-16E331D6D3BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3152DB39-93A4-41FB-8D06-E7A5841EA1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1905" windowWidth="29040" windowHeight="17520" xr2:uid="{8BCFAE85-CB20-435D-AEB6-6494F3D318DE}"/>
+    <workbookView minimized="1" xWindow="5268" yWindow="3564" windowWidth="17280" windowHeight="8880" xr2:uid="{8BCFAE85-CB20-435D-AEB6-6494F3D318DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -783,47 +783,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="85">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="81">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1971,8 +1931,8 @@
     <col min="2" max="2" width="94" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.59765625" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="6.8984375" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="25" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="24.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.8984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6025,165 +5985,165 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1">
-    <cfRule type="duplicateValues" dxfId="84" priority="79"/>
-    <cfRule type="duplicateValues" dxfId="83" priority="80"/>
-    <cfRule type="duplicateValues" dxfId="82" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B134">
-    <cfRule type="duplicateValues" dxfId="81" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B3">
-    <cfRule type="duplicateValues" dxfId="80" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="76"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B13">
-    <cfRule type="duplicateValues" dxfId="79" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="74"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B35">
-    <cfRule type="duplicateValues" dxfId="78" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4">
-    <cfRule type="duplicateValues" dxfId="77" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="75"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:B6">
-    <cfRule type="duplicateValues" dxfId="76" priority="77"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:B10">
-    <cfRule type="duplicateValues" dxfId="75" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="78"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:B13">
-    <cfRule type="duplicateValues" dxfId="74" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:B35">
-    <cfRule type="duplicateValues" dxfId="73" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B36:B55">
-    <cfRule type="duplicateValues" dxfId="72" priority="69"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="70"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B56">
-    <cfRule type="duplicateValues" dxfId="70" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B57:B58">
-    <cfRule type="duplicateValues" dxfId="69" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59:B60">
-    <cfRule type="duplicateValues" dxfId="68" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B61">
-    <cfRule type="duplicateValues" dxfId="67" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B62:B90">
-    <cfRule type="duplicateValues" dxfId="66" priority="62"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="63"/>
-    <cfRule type="duplicateValues" dxfId="64" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B91:B92">
-    <cfRule type="duplicateValues" dxfId="63" priority="55"/>
-    <cfRule type="duplicateValues" dxfId="62" priority="56"/>
-    <cfRule type="duplicateValues" dxfId="61" priority="57"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="58"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93:B94">
-    <cfRule type="duplicateValues" dxfId="59" priority="53"/>
-    <cfRule type="duplicateValues" dxfId="58" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95:B134">
-    <cfRule type="duplicateValues" dxfId="57" priority="50"/>
-    <cfRule type="duplicateValues" dxfId="56" priority="51"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B135:B164">
-    <cfRule type="duplicateValues" dxfId="54" priority="47"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B165">
-    <cfRule type="duplicateValues" dxfId="52" priority="43"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="44"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="45"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="46"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B90">
-    <cfRule type="duplicateValues" dxfId="48" priority="59"/>
-    <cfRule type="duplicateValues" dxfId="47" priority="60"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="61"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="45" priority="40"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="41"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="42" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="41" priority="37"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="38"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="38" priority="33"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="34"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="35" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="34" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="31"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="31" priority="26"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="27"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="28" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="27" priority="23"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="24"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="duplicateValues" dxfId="24" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="duplicateValues" dxfId="21" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="17"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1">
-    <cfRule type="duplicateValues" dxfId="17" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1">
-    <cfRule type="duplicateValues" dxfId="14" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1">
-    <cfRule type="duplicateValues" dxfId="13" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1">
-    <cfRule type="duplicateValues" dxfId="10" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1">
-    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1">
-    <cfRule type="duplicateValues" dxfId="6" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>